<commit_message>
fix: mcps y caja de prompts
</commit_message>
<xml_diff>
--- a/storage/workspaces/facturas/documents/facturas_450_filas.xlsx
+++ b/storage/workspaces/facturas/documents/facturas_450_filas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\Proyectos\3 - AI_KnowledgeHub\AI_KnowledgeHub\storage\workspaces\facturas\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35633E19-7D4D-4A25-BA46-63D9C62401F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED207BE-E356-44CE-B827-8AA53E900F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6785" uniqueCount="3724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6935" uniqueCount="3724">
   <si>
     <t>Emisor_mail</t>
   </si>
@@ -11559,7 +11559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AI451"/>
+  <dimension ref="A1:AI461"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
@@ -40919,6 +40919,656 @@
         <v>3722</v>
       </c>
     </row>
+    <row r="452" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A452" t="s">
+        <v>431</v>
+      </c>
+      <c r="B452" t="s">
+        <v>513</v>
+      </c>
+      <c r="C452" t="s">
+        <v>911</v>
+      </c>
+      <c r="F452" t="s">
+        <v>1361</v>
+      </c>
+      <c r="G452" t="s">
+        <v>1721</v>
+      </c>
+      <c r="H452">
+        <v>24695195461</v>
+      </c>
+      <c r="I452" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K452" t="s">
+        <v>2151</v>
+      </c>
+      <c r="L452">
+        <v>25888624403</v>
+      </c>
+      <c r="M452" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O452" t="s">
+        <v>2601</v>
+      </c>
+      <c r="P452" t="s">
+        <v>3051</v>
+      </c>
+      <c r="Q452" t="s">
+        <v>3501</v>
+      </c>
+      <c r="R452">
+        <v>542153.16</v>
+      </c>
+      <c r="Y452">
+        <v>32200775574340</v>
+      </c>
+      <c r="Z452" t="s">
+        <v>3702</v>
+      </c>
+      <c r="AB452">
+        <v>542153.16</v>
+      </c>
+      <c r="AD452" t="s">
+        <v>3719</v>
+      </c>
+      <c r="AF452" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AH452">
+        <v>25888624403</v>
+      </c>
+      <c r="AI452" t="s">
+        <v>3722</v>
+      </c>
+    </row>
+    <row r="453" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A453" t="s">
+        <v>432</v>
+      </c>
+      <c r="B453" t="s">
+        <v>504</v>
+      </c>
+      <c r="C453" t="s">
+        <v>912</v>
+      </c>
+      <c r="F453" t="s">
+        <v>1362</v>
+      </c>
+      <c r="G453" t="s">
+        <v>1584</v>
+      </c>
+      <c r="H453">
+        <v>25558175597</v>
+      </c>
+      <c r="I453" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K453" t="s">
+        <v>2152</v>
+      </c>
+      <c r="L453">
+        <v>28979346307</v>
+      </c>
+      <c r="M453" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O453" t="s">
+        <v>2602</v>
+      </c>
+      <c r="P453" t="s">
+        <v>3052</v>
+      </c>
+      <c r="Q453" t="s">
+        <v>3502</v>
+      </c>
+      <c r="R453">
+        <v>458122.26</v>
+      </c>
+      <c r="Y453">
+        <v>54796183870355</v>
+      </c>
+      <c r="Z453" t="s">
+        <v>1648</v>
+      </c>
+      <c r="AB453">
+        <v>458122.26</v>
+      </c>
+      <c r="AD453" t="s">
+        <v>3719</v>
+      </c>
+      <c r="AF453" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AH453">
+        <v>28979346307</v>
+      </c>
+      <c r="AI453" t="s">
+        <v>3723</v>
+      </c>
+    </row>
+    <row r="454" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A454" t="s">
+        <v>433</v>
+      </c>
+      <c r="B454" t="s">
+        <v>489</v>
+      </c>
+      <c r="C454" t="s">
+        <v>913</v>
+      </c>
+      <c r="F454" t="s">
+        <v>1363</v>
+      </c>
+      <c r="G454" t="s">
+        <v>1688</v>
+      </c>
+      <c r="H454">
+        <v>26154240534</v>
+      </c>
+      <c r="I454" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K454" t="s">
+        <v>2153</v>
+      </c>
+      <c r="L454">
+        <v>22526205273</v>
+      </c>
+      <c r="M454" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O454" t="s">
+        <v>2603</v>
+      </c>
+      <c r="P454" t="s">
+        <v>3053</v>
+      </c>
+      <c r="Q454" t="s">
+        <v>3503</v>
+      </c>
+      <c r="R454">
+        <v>165834.78</v>
+      </c>
+      <c r="Y454">
+        <v>81873635133592</v>
+      </c>
+      <c r="Z454" t="s">
+        <v>3703</v>
+      </c>
+      <c r="AB454">
+        <v>165834.78</v>
+      </c>
+      <c r="AD454" t="s">
+        <v>3719</v>
+      </c>
+      <c r="AF454" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AH454">
+        <v>22526205273</v>
+      </c>
+      <c r="AI454" t="s">
+        <v>3723</v>
+      </c>
+    </row>
+    <row r="455" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A455" t="s">
+        <v>434</v>
+      </c>
+      <c r="B455" t="s">
+        <v>495</v>
+      </c>
+      <c r="C455" t="s">
+        <v>914</v>
+      </c>
+      <c r="F455" t="s">
+        <v>1364</v>
+      </c>
+      <c r="G455" t="s">
+        <v>1608</v>
+      </c>
+      <c r="H455">
+        <v>20998628965</v>
+      </c>
+      <c r="I455" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K455" t="s">
+        <v>2154</v>
+      </c>
+      <c r="L455">
+        <v>29274265918</v>
+      </c>
+      <c r="M455" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O455" t="s">
+        <v>2604</v>
+      </c>
+      <c r="P455" t="s">
+        <v>3054</v>
+      </c>
+      <c r="Q455" t="s">
+        <v>3504</v>
+      </c>
+      <c r="R455">
+        <v>453277.42</v>
+      </c>
+      <c r="Y455">
+        <v>87514660146922</v>
+      </c>
+      <c r="Z455" t="s">
+        <v>1746</v>
+      </c>
+      <c r="AB455">
+        <v>453277.42</v>
+      </c>
+      <c r="AD455" t="s">
+        <v>3719</v>
+      </c>
+      <c r="AF455" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AH455">
+        <v>29274265918</v>
+      </c>
+      <c r="AI455" t="s">
+        <v>3722</v>
+      </c>
+    </row>
+    <row r="456" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A456" t="s">
+        <v>435</v>
+      </c>
+      <c r="B456" t="s">
+        <v>500</v>
+      </c>
+      <c r="C456" t="s">
+        <v>915</v>
+      </c>
+      <c r="F456" t="s">
+        <v>1365</v>
+      </c>
+      <c r="G456" t="s">
+        <v>1536</v>
+      </c>
+      <c r="H456">
+        <v>26224926428</v>
+      </c>
+      <c r="I456" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K456" t="s">
+        <v>2155</v>
+      </c>
+      <c r="L456">
+        <v>30697410236</v>
+      </c>
+      <c r="M456" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O456" t="s">
+        <v>2605</v>
+      </c>
+      <c r="P456" t="s">
+        <v>3055</v>
+      </c>
+      <c r="Q456" t="s">
+        <v>3505</v>
+      </c>
+      <c r="R456">
+        <v>370479.11</v>
+      </c>
+      <c r="Y456">
+        <v>17010902820873</v>
+      </c>
+      <c r="Z456" t="s">
+        <v>1534</v>
+      </c>
+      <c r="AB456">
+        <v>370479.11</v>
+      </c>
+      <c r="AD456" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AF456" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AH456">
+        <v>30697410236</v>
+      </c>
+      <c r="AI456" t="s">
+        <v>3723</v>
+      </c>
+    </row>
+    <row r="457" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A457" t="s">
+        <v>436</v>
+      </c>
+      <c r="B457" t="s">
+        <v>492</v>
+      </c>
+      <c r="C457" t="s">
+        <v>916</v>
+      </c>
+      <c r="F457" t="s">
+        <v>1366</v>
+      </c>
+      <c r="G457" t="s">
+        <v>1722</v>
+      </c>
+      <c r="H457">
+        <v>30700976669</v>
+      </c>
+      <c r="I457" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K457" t="s">
+        <v>2156</v>
+      </c>
+      <c r="L457">
+        <v>28221113366</v>
+      </c>
+      <c r="M457" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O457" t="s">
+        <v>2606</v>
+      </c>
+      <c r="P457" t="s">
+        <v>3056</v>
+      </c>
+      <c r="Q457" t="s">
+        <v>3506</v>
+      </c>
+      <c r="R457">
+        <v>443557.15</v>
+      </c>
+      <c r="Y457">
+        <v>70620068733142</v>
+      </c>
+      <c r="Z457" t="s">
+        <v>3704</v>
+      </c>
+      <c r="AB457">
+        <v>443557.15</v>
+      </c>
+      <c r="AD457" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AF457" t="s">
+        <v>3719</v>
+      </c>
+      <c r="AH457">
+        <v>28221113366</v>
+      </c>
+      <c r="AI457" t="s">
+        <v>3723</v>
+      </c>
+    </row>
+    <row r="458" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A458" t="s">
+        <v>437</v>
+      </c>
+      <c r="B458" t="s">
+        <v>500</v>
+      </c>
+      <c r="C458" t="s">
+        <v>917</v>
+      </c>
+      <c r="F458" t="s">
+        <v>1367</v>
+      </c>
+      <c r="G458" t="s">
+        <v>1723</v>
+      </c>
+      <c r="H458">
+        <v>27711760429</v>
+      </c>
+      <c r="I458" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K458" t="s">
+        <v>2157</v>
+      </c>
+      <c r="L458">
+        <v>20439754700</v>
+      </c>
+      <c r="M458" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O458" t="s">
+        <v>2607</v>
+      </c>
+      <c r="P458" t="s">
+        <v>3057</v>
+      </c>
+      <c r="Q458" t="s">
+        <v>3507</v>
+      </c>
+      <c r="R458">
+        <v>187686.76</v>
+      </c>
+      <c r="Y458">
+        <v>30810795018270</v>
+      </c>
+      <c r="Z458" t="s">
+        <v>3683</v>
+      </c>
+      <c r="AB458">
+        <v>187686.76</v>
+      </c>
+      <c r="AD458" t="s">
+        <v>3719</v>
+      </c>
+      <c r="AF458" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AH458">
+        <v>20439754700</v>
+      </c>
+      <c r="AI458" t="s">
+        <v>3723</v>
+      </c>
+    </row>
+    <row r="459" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A459" t="s">
+        <v>438</v>
+      </c>
+      <c r="B459" t="s">
+        <v>508</v>
+      </c>
+      <c r="C459" t="s">
+        <v>918</v>
+      </c>
+      <c r="F459" t="s">
+        <v>1368</v>
+      </c>
+      <c r="G459" t="s">
+        <v>1724</v>
+      </c>
+      <c r="H459">
+        <v>30943852507</v>
+      </c>
+      <c r="I459" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K459" t="s">
+        <v>2158</v>
+      </c>
+      <c r="L459">
+        <v>29800804458</v>
+      </c>
+      <c r="M459" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O459" t="s">
+        <v>2608</v>
+      </c>
+      <c r="P459" t="s">
+        <v>3058</v>
+      </c>
+      <c r="Q459" t="s">
+        <v>3508</v>
+      </c>
+      <c r="R459">
+        <v>95310.68</v>
+      </c>
+      <c r="Y459">
+        <v>33197736026072</v>
+      </c>
+      <c r="Z459" t="s">
+        <v>1567</v>
+      </c>
+      <c r="AB459">
+        <v>95310.68</v>
+      </c>
+      <c r="AD459" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AF459" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AH459">
+        <v>29800804458</v>
+      </c>
+      <c r="AI459" t="s">
+        <v>3721</v>
+      </c>
+    </row>
+    <row r="460" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A460" t="s">
+        <v>439</v>
+      </c>
+      <c r="B460" t="s">
+        <v>506</v>
+      </c>
+      <c r="C460" t="s">
+        <v>919</v>
+      </c>
+      <c r="F460" t="s">
+        <v>1369</v>
+      </c>
+      <c r="G460" t="s">
+        <v>1725</v>
+      </c>
+      <c r="H460">
+        <v>30540474257</v>
+      </c>
+      <c r="I460" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K460" t="s">
+        <v>2159</v>
+      </c>
+      <c r="L460">
+        <v>23675193453</v>
+      </c>
+      <c r="M460" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O460" t="s">
+        <v>2609</v>
+      </c>
+      <c r="P460" t="s">
+        <v>3059</v>
+      </c>
+      <c r="Q460" t="s">
+        <v>3509</v>
+      </c>
+      <c r="R460">
+        <v>241119.82</v>
+      </c>
+      <c r="Y460">
+        <v>24689506209336</v>
+      </c>
+      <c r="Z460" t="s">
+        <v>1545</v>
+      </c>
+      <c r="AB460">
+        <v>241119.82</v>
+      </c>
+      <c r="AD460" t="s">
+        <v>3719</v>
+      </c>
+      <c r="AF460" t="s">
+        <v>3719</v>
+      </c>
+      <c r="AH460">
+        <v>23675193453</v>
+      </c>
+      <c r="AI460" t="s">
+        <v>3723</v>
+      </c>
+    </row>
+    <row r="461" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A461" t="s">
+        <v>440</v>
+      </c>
+      <c r="B461" t="s">
+        <v>505</v>
+      </c>
+      <c r="C461" t="s">
+        <v>920</v>
+      </c>
+      <c r="F461" t="s">
+        <v>1370</v>
+      </c>
+      <c r="G461" t="s">
+        <v>1726</v>
+      </c>
+      <c r="H461">
+        <v>25378761984</v>
+      </c>
+      <c r="I461" t="s">
+        <v>1754</v>
+      </c>
+      <c r="K461" t="s">
+        <v>2160</v>
+      </c>
+      <c r="L461">
+        <v>27702353678</v>
+      </c>
+      <c r="M461" t="s">
+        <v>1754</v>
+      </c>
+      <c r="O461" t="s">
+        <v>2610</v>
+      </c>
+      <c r="P461" t="s">
+        <v>3060</v>
+      </c>
+      <c r="Q461" t="s">
+        <v>3510</v>
+      </c>
+      <c r="R461">
+        <v>830570.05</v>
+      </c>
+      <c r="Y461">
+        <v>16846739564402</v>
+      </c>
+      <c r="Z461" t="s">
+        <v>1544</v>
+      </c>
+      <c r="AB461">
+        <v>830570.05</v>
+      </c>
+      <c r="AD461" t="s">
+        <v>3720</v>
+      </c>
+      <c r="AF461" t="s">
+        <v>3719</v>
+      </c>
+      <c r="AH461">
+        <v>27702353678</v>
+      </c>
+      <c r="AI461" t="s">
+        <v>3722</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>